<commit_message>
docs(fase11): figuras regeneradas, benchmark por selección de redes, capturas GUI, fecha sin datetime2
- Figuras estáticas (9) e interactivas (8) regeneradas desde benchmark.csv actual;
  make_interactive con orden de imports arreglado; ambos apuntan a benchmark.csv.
- GUI: el benchmark ahora deja elegir qué redes de data/samples/ incluir (multiselect
  + Generar/Regenerar) en vez de N10A fijo.
- Manual_Usuario: 4 capturas reales de la GUI vía \guishot/\IfFileExists (generar TPM,
  ejecución k3/N10A, tabla de evaluación, benchmark N20A con selector de redes);
  data/.screenshots/ en .gitignore.
- preambulo: fecha personalizada reimplementada como \mesano (sin datetime2/tracklang
  ausente) y enlazada en ambas portadas. make all en verde: 21 + 11 = 32 páginas.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/results/benchmark.xlsx
+++ b/data/results/benchmark.xlsx
@@ -480,7 +480,7 @@
         <v>0.469727</v>
       </c>
       <c r="F2" t="n">
-        <v>0.0168</v>
+        <v>0.0224</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
@@ -511,7 +511,7 @@
         <v>0.469727</v>
       </c>
       <c r="F3" t="n">
-        <v>0.1113</v>
+        <v>0.1192</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
@@ -542,7 +542,7 @@
         <v>4.6875</v>
       </c>
       <c r="F4" t="n">
-        <v>0.0061</v>
+        <v>0.0131</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
@@ -573,7 +573,7 @@
         <v>4.734375</v>
       </c>
       <c r="F5" t="n">
-        <v>0.0041</v>
+        <v>0.0065</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
@@ -604,7 +604,7 @@
         <v>0.469727</v>
       </c>
       <c r="F6" t="n">
-        <v>0.8536</v>
+        <v>0.7027</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
@@ -635,7 +635,7 @@
         <v>0.472656</v>
       </c>
       <c r="F7" t="n">
-        <v>0.2247</v>
+        <v>0.2817</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
@@ -666,7 +666,7 @@
         <v>0.469727</v>
       </c>
       <c r="F8" t="n">
-        <v>0.8685</v>
+        <v>0.7256</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
@@ -697,7 +697,7 @@
         <v>0.942383</v>
       </c>
       <c r="F9" t="n">
-        <v>0.0296</v>
+        <v>0.0327</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
@@ -729,7 +729,7 @@
         <v>0.942383</v>
       </c>
       <c r="F10" t="n">
-        <v>0.1194</v>
+        <v>0.1283</v>
       </c>
       <c r="G10" t="inlineStr">
         <is>
@@ -761,7 +761,7 @@
         <v>4.871094</v>
       </c>
       <c r="F11" t="n">
-        <v>0.005</v>
+        <v>0.0052</v>
       </c>
       <c r="G11" t="inlineStr">
         <is>
@@ -793,7 +793,7 @@
         <v>4.863281</v>
       </c>
       <c r="F12" t="n">
-        <v>0.0039</v>
+        <v>0.0047</v>
       </c>
       <c r="G12" t="inlineStr">
         <is>
@@ -825,7 +825,7 @@
         <v>0.958008</v>
       </c>
       <c r="F13" t="n">
-        <v>1.6009</v>
+        <v>1.3413</v>
       </c>
       <c r="G13" t="inlineStr">
         <is>
@@ -857,7 +857,7 @@
         <v>0.963867</v>
       </c>
       <c r="F14" t="n">
-        <v>0.7419</v>
+        <v>0.6691</v>
       </c>
       <c r="G14" t="inlineStr">
         <is>
@@ -889,7 +889,7 @@
         <v>0.942383</v>
       </c>
       <c r="F15" t="n">
-        <v>1.6552</v>
+        <v>1.5857</v>
       </c>
       <c r="G15" t="inlineStr">
         <is>
@@ -921,7 +921,7 @@
         <v>1.422852</v>
       </c>
       <c r="F16" t="n">
-        <v>0.07389999999999999</v>
+        <v>0.0395</v>
       </c>
       <c r="G16" t="inlineStr">
         <is>
@@ -954,7 +954,7 @@
         <v>1.422852</v>
       </c>
       <c r="F17" t="n">
-        <v>0.2406</v>
+        <v>0.1388</v>
       </c>
       <c r="G17" t="inlineStr">
         <is>
@@ -987,7 +987,7 @@
         <v>5.007812</v>
       </c>
       <c r="F18" t="n">
-        <v>0.0119</v>
+        <v>0.0049</v>
       </c>
       <c r="G18" t="inlineStr">
         <is>
@@ -1020,7 +1020,7 @@
         <v>5.011719</v>
       </c>
       <c r="F19" t="n">
-        <v>0.008</v>
+        <v>0.0049</v>
       </c>
       <c r="G19" t="inlineStr">
         <is>
@@ -1053,7 +1053,7 @@
         <v>2.391602</v>
       </c>
       <c r="F20" t="n">
-        <v>1.1594</v>
+        <v>1.0782</v>
       </c>
       <c r="G20" t="inlineStr">
         <is>
@@ -1086,7 +1086,7 @@
         <v>1.436523</v>
       </c>
       <c r="F21" t="n">
-        <v>0.8642</v>
+        <v>0.7713</v>
       </c>
       <c r="G21" t="inlineStr">
         <is>
@@ -1119,7 +1119,7 @@
         <v>1.422852</v>
       </c>
       <c r="F22" t="n">
-        <v>2.1898</v>
+        <v>2.3047</v>
       </c>
       <c r="G22" t="inlineStr">
         <is>
@@ -1152,7 +1152,7 @@
         <v>1.911133</v>
       </c>
       <c r="F23" t="n">
-        <v>0.0434</v>
+        <v>0.0536</v>
       </c>
       <c r="G23" t="inlineStr">
         <is>
@@ -1186,7 +1186,7 @@
         <v>1.911133</v>
       </c>
       <c r="F24" t="n">
-        <v>0.1292</v>
+        <v>0.1633</v>
       </c>
       <c r="G24" t="inlineStr">
         <is>
@@ -1220,7 +1220,7 @@
         <v>4.851562</v>
       </c>
       <c r="F25" t="n">
-        <v>0.0077</v>
+        <v>0.0048</v>
       </c>
       <c r="G25" t="inlineStr">
         <is>
@@ -1254,7 +1254,7 @@
         <v>4.992188</v>
       </c>
       <c r="F26" t="n">
-        <v>0.0078</v>
+        <v>0.008200000000000001</v>
       </c>
       <c r="G26" t="inlineStr">
         <is>
@@ -1288,7 +1288,7 @@
         <v>1.938477</v>
       </c>
       <c r="F27" t="n">
-        <v>1.7731</v>
+        <v>1.7161</v>
       </c>
       <c r="G27" t="inlineStr">
         <is>
@@ -1322,7 +1322,7 @@
         <v>1.975586</v>
       </c>
       <c r="F28" t="n">
-        <v>1.0129</v>
+        <v>1.0419</v>
       </c>
       <c r="G28" t="inlineStr">
         <is>
@@ -1356,7 +1356,7 @@
         <v>1.911133</v>
       </c>
       <c r="F29" t="n">
-        <v>2.5465</v>
+        <v>5.1986</v>
       </c>
       <c r="G29" t="inlineStr">
         <is>
@@ -1390,7 +1390,7 @@
         <v>0.02679</v>
       </c>
       <c r="F30" t="n">
-        <v>0.0605</v>
+        <v>0.2921</v>
       </c>
       <c r="G30" t="inlineStr">
         <is>
@@ -1421,7 +1421,7 @@
         <v>0.02679</v>
       </c>
       <c r="F31" t="n">
-        <v>0.6259</v>
+        <v>1.4848</v>
       </c>
       <c r="G31" t="inlineStr">
         <is>
@@ -1452,7 +1452,7 @@
         <v>0.527377</v>
       </c>
       <c r="F32" t="n">
-        <v>0.0177</v>
+        <v>0.022</v>
       </c>
       <c r="G32" t="inlineStr">
         <is>
@@ -1483,7 +1483,7 @@
         <v>0.527377</v>
       </c>
       <c r="F33" t="n">
-        <v>0.0295</v>
+        <v>0.0344</v>
       </c>
       <c r="G33" t="inlineStr">
         <is>
@@ -1514,7 +1514,7 @@
         <v>0.027029</v>
       </c>
       <c r="F34" t="n">
-        <v>1.361</v>
+        <v>3.1821</v>
       </c>
       <c r="G34" t="inlineStr">
         <is>
@@ -1545,7 +1545,7 @@
         <v>0.027127</v>
       </c>
       <c r="F35" t="n">
-        <v>0.9416</v>
+        <v>2.0781</v>
       </c>
       <c r="G35" t="inlineStr">
         <is>
@@ -1576,7 +1576,7 @@
         <v>0.02679</v>
       </c>
       <c r="F36" t="n">
-        <v>1.7978</v>
+        <v>2.5708</v>
       </c>
       <c r="G36" t="inlineStr">
         <is>
@@ -1607,7 +1607,7 @@
         <v>0.053819</v>
       </c>
       <c r="F37" t="n">
-        <v>0.08550000000000001</v>
+        <v>0.2502</v>
       </c>
       <c r="G37" t="inlineStr">
         <is>
@@ -1639,7 +1639,7 @@
         <v>0.053899</v>
       </c>
       <c r="F38" t="n">
-        <v>0.7044</v>
+        <v>1.0513</v>
       </c>
       <c r="G38" t="inlineStr">
         <is>
@@ -1671,7 +1671,7 @@
         <v>0.875242</v>
       </c>
       <c r="F39" t="n">
-        <v>0.009299999999999999</v>
+        <v>0.0162</v>
       </c>
       <c r="G39" t="inlineStr">
         <is>
@@ -1703,7 +1703,7 @@
         <v>1.07105</v>
       </c>
       <c r="F40" t="n">
-        <v>0.0112</v>
+        <v>0.0182</v>
       </c>
       <c r="G40" t="inlineStr">
         <is>
@@ -1735,7 +1735,7 @@
         <v>0.053899</v>
       </c>
       <c r="F41" t="n">
-        <v>1.6002</v>
+        <v>2.7499</v>
       </c>
       <c r="G41" t="inlineStr">
         <is>
@@ -1767,7 +1767,7 @@
         <v>0.054019</v>
       </c>
       <c r="F42" t="n">
-        <v>1.4202</v>
+        <v>1.9823</v>
       </c>
       <c r="G42" t="inlineStr">
         <is>
@@ -1799,7 +1799,7 @@
         <v>0.053819</v>
       </c>
       <c r="F43" t="n">
-        <v>2.8475</v>
+        <v>4.4157</v>
       </c>
       <c r="G43" t="inlineStr">
         <is>
@@ -1831,7 +1831,7 @@
         <v>0.080928</v>
       </c>
       <c r="F44" t="n">
-        <v>0.1018</v>
+        <v>0.2358</v>
       </c>
       <c r="G44" t="inlineStr">
         <is>
@@ -1864,7 +1864,7 @@
         <v>0.081027</v>
       </c>
       <c r="F45" t="n">
-        <v>0.6767</v>
+        <v>0.7759</v>
       </c>
       <c r="G45" t="inlineStr">
         <is>
@@ -1897,7 +1897,7 @@
         <v>1.055199</v>
       </c>
       <c r="F46" t="n">
-        <v>0.008699999999999999</v>
+        <v>0.0108</v>
       </c>
       <c r="G46" t="inlineStr">
         <is>
@@ -1930,7 +1930,7 @@
         <v>1.076201</v>
       </c>
       <c r="F47" t="n">
-        <v>0.0111</v>
+        <v>0.0094</v>
       </c>
       <c r="G47" t="inlineStr">
         <is>
@@ -1963,7 +1963,7 @@
         <v>0.833143</v>
       </c>
       <c r="F48" t="n">
-        <v>2.9904</v>
+        <v>3.7845</v>
       </c>
       <c r="G48" t="inlineStr">
         <is>
@@ -1996,7 +1996,7 @@
         <v>0.834553</v>
       </c>
       <c r="F49" t="n">
-        <v>1.879</v>
+        <v>1.4305</v>
       </c>
       <c r="G49" t="inlineStr">
         <is>
@@ -2029,7 +2029,7 @@
         <v>0.08094700000000001</v>
       </c>
       <c r="F50" t="n">
-        <v>3.9927</v>
+        <v>3.0532</v>
       </c>
       <c r="G50" t="inlineStr">
         <is>
@@ -2062,7 +2062,7 @@
         <v>0.108056</v>
       </c>
       <c r="F51" t="n">
-        <v>0.2069</v>
+        <v>0.1221</v>
       </c>
       <c r="G51" t="inlineStr">
         <is>
@@ -2096,7 +2096,7 @@
         <v>0.10818</v>
       </c>
       <c r="F52" t="n">
-        <v>0.7415</v>
+        <v>0.6183999999999999</v>
       </c>
       <c r="G52" t="inlineStr">
         <is>
@@ -2130,7 +2130,7 @@
         <v>1.089651</v>
       </c>
       <c r="F53" t="n">
-        <v>0.0072</v>
+        <v>0.0091</v>
       </c>
       <c r="G53" t="inlineStr">
         <is>
@@ -2164,7 +2164,7 @@
         <v>1.082651</v>
       </c>
       <c r="F54" t="n">
-        <v>0.008500000000000001</v>
+        <v>0.0089</v>
       </c>
       <c r="G54" t="inlineStr">
         <is>
@@ -2198,7 +2198,7 @@
         <v>0.108056</v>
       </c>
       <c r="F55" t="n">
-        <v>3.6988</v>
+        <v>3.2998</v>
       </c>
       <c r="G55" t="inlineStr">
         <is>
@@ -2232,7 +2232,7 @@
         <v>0.88572</v>
       </c>
       <c r="F56" t="n">
-        <v>2.7966</v>
+        <v>1.5497</v>
       </c>
       <c r="G56" t="inlineStr">
         <is>
@@ -2266,7 +2266,7 @@
         <v>0.108056</v>
       </c>
       <c r="F57" t="n">
-        <v>3.8865</v>
+        <v>3.0202</v>
       </c>
       <c r="G57" t="inlineStr">
         <is>
@@ -2300,7 +2300,7 @@
         <v>0.499296</v>
       </c>
       <c r="F58" t="n">
-        <v>4.317</v>
+        <v>2.3524</v>
       </c>
       <c r="G58" t="inlineStr">
         <is>
@@ -2331,7 +2331,7 @@
         <v>0.499296</v>
       </c>
       <c r="F59" t="n">
-        <v>6.2692</v>
+        <v>2.4145</v>
       </c>
       <c r="G59" t="inlineStr">
         <is>
@@ -2362,7 +2362,7 @@
         <v>9.988281000000001</v>
       </c>
       <c r="F60" t="n">
-        <v>0.164</v>
+        <v>0.0746</v>
       </c>
       <c r="G60" t="inlineStr">
         <is>
@@ -2393,7 +2393,7 @@
         <v>10.064453</v>
       </c>
       <c r="F61" t="n">
-        <v>0.1375</v>
+        <v>0.0868</v>
       </c>
       <c r="G61" t="inlineStr">
         <is>
@@ -2424,7 +2424,7 @@
         <v>0.499296</v>
       </c>
       <c r="F62" t="n">
-        <v>7.5422</v>
+        <v>3.6729</v>
       </c>
       <c r="G62" t="inlineStr">
         <is>
@@ -2455,7 +2455,7 @@
         <v>0.499616</v>
       </c>
       <c r="F63" t="n">
-        <v>4.1483</v>
+        <v>2.5356</v>
       </c>
       <c r="G63" t="inlineStr">
         <is>
@@ -2486,7 +2486,7 @@
         <v>0.499296</v>
       </c>
       <c r="F64" t="n">
-        <v>5.6706</v>
+        <v>3.8633</v>
       </c>
       <c r="G64" t="inlineStr">
         <is>
@@ -2517,7 +2517,7 @@
         <v>0.998684</v>
       </c>
       <c r="F65" t="n">
-        <v>5.5044</v>
+        <v>3.7949</v>
       </c>
       <c r="G65" t="inlineStr">
         <is>
@@ -2549,7 +2549,7 @@
         <v>0.998684</v>
       </c>
       <c r="F66" t="n">
-        <v>7.8903</v>
+        <v>2.9021</v>
       </c>
       <c r="G66" t="inlineStr">
         <is>
@@ -2581,7 +2581,7 @@
         <v>10.019196</v>
       </c>
       <c r="F67" t="n">
-        <v>0.2869</v>
+        <v>0.1231</v>
       </c>
       <c r="G67" t="inlineStr">
         <is>
@@ -2613,7 +2613,7 @@
         <v>10.059732</v>
       </c>
       <c r="F68" t="n">
-        <v>0.3211</v>
+        <v>0.107</v>
       </c>
       <c r="G68" t="inlineStr">
         <is>
@@ -2645,7 +2645,7 @@
         <v>1.499331</v>
       </c>
       <c r="F69" t="n">
-        <v>11.4141</v>
+        <v>6.036</v>
       </c>
       <c r="G69" t="inlineStr">
         <is>
@@ -2677,7 +2677,7 @@
         <v>1.00018</v>
       </c>
       <c r="F70" t="n">
-        <v>4.8139</v>
+        <v>2.5336</v>
       </c>
       <c r="G70" t="inlineStr">
         <is>
@@ -2709,7 +2709,7 @@
         <v>0.998684</v>
       </c>
       <c r="F71" t="n">
-        <v>7.0729</v>
+        <v>4.5767</v>
       </c>
       <c r="G71" t="inlineStr">
         <is>
@@ -2741,7 +2741,7 @@
         <v>1.498185</v>
       </c>
       <c r="F72" t="n">
-        <v>5.0663</v>
+        <v>4.0675</v>
       </c>
       <c r="G72" t="inlineStr">
         <is>
@@ -2774,7 +2774,7 @@
         <v>1.498185</v>
       </c>
       <c r="F73" t="n">
-        <v>5.0106</v>
+        <v>3.0636</v>
       </c>
       <c r="G73" t="inlineStr">
         <is>
@@ -2807,7 +2807,7 @@
         <v>10.022339</v>
       </c>
       <c r="F74" t="n">
-        <v>0.2541</v>
+        <v>0.08160000000000001</v>
       </c>
       <c r="G74" t="inlineStr">
         <is>
@@ -2840,7 +2840,7 @@
         <v>10.055605</v>
       </c>
       <c r="F75" t="n">
-        <v>0.2452</v>
+        <v>0.1081</v>
       </c>
       <c r="G75" t="inlineStr">
         <is>
@@ -2873,7 +2873,7 @@
         <v>3.998016</v>
       </c>
       <c r="F76" t="n">
-        <v>10.999</v>
+        <v>8.188499999999999</v>
       </c>
       <c r="G76" t="inlineStr">
         <is>
@@ -2906,7 +2906,7 @@
         <v>6.999811</v>
       </c>
       <c r="F77" t="n">
-        <v>4.4538</v>
+        <v>3.5016</v>
       </c>
       <c r="G77" t="inlineStr">
         <is>
@@ -2939,7 +2939,7 @@
         <v>1.498507</v>
       </c>
       <c r="F78" t="n">
-        <v>6.5053</v>
+        <v>4.907</v>
       </c>
       <c r="G78" t="inlineStr">
         <is>
@@ -2972,7 +2972,7 @@
         <v>1.997801</v>
       </c>
       <c r="F79" t="n">
-        <v>5.1462</v>
+        <v>4.607</v>
       </c>
       <c r="G79" t="inlineStr">
         <is>
@@ -3006,7 +3006,7 @@
         <v>1.997801</v>
       </c>
       <c r="F80" t="n">
-        <v>4.2065</v>
+        <v>6.8455</v>
       </c>
       <c r="G80" t="inlineStr">
         <is>
@@ -3040,7 +3040,7 @@
         <v>10.009598</v>
       </c>
       <c r="F81" t="n">
-        <v>0.1296</v>
+        <v>0.2411</v>
       </c>
       <c r="G81" t="inlineStr">
         <is>
@@ -3074,7 +3074,7 @@
         <v>10.011873</v>
       </c>
       <c r="F82" t="n">
-        <v>0.1057</v>
+        <v>0.2509</v>
       </c>
       <c r="G82" t="inlineStr">
         <is>
@@ -3108,7 +3108,7 @@
         <v>4.997678</v>
       </c>
       <c r="F83" t="n">
-        <v>10.2392</v>
+        <v>12.3664</v>
       </c>
       <c r="G83" t="inlineStr">
         <is>
@@ -3142,7 +3142,7 @@
         <v>5.497547</v>
       </c>
       <c r="F84" t="n">
-        <v>4.7448</v>
+        <v>6.1723</v>
       </c>
       <c r="G84" t="inlineStr">
         <is>
@@ -3176,7 +3176,7 @@
         <v>1.997874</v>
       </c>
       <c r="F85" t="n">
-        <v>6.6537</v>
+        <v>5.681</v>
       </c>
       <c r="G85" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
docs: manual técnico y usuario — referencias, pseudocódigo, limpieza
</commit_message>
<xml_diff>
--- a/data/results/benchmark.xlsx
+++ b/data/results/benchmark.xlsx
@@ -480,7 +480,7 @@
         <v>0.469727</v>
       </c>
       <c r="F2" t="n">
-        <v>0.0224</v>
+        <v>0.0137</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
@@ -511,7 +511,7 @@
         <v>0.469727</v>
       </c>
       <c r="F3" t="n">
-        <v>0.1192</v>
+        <v>0.0698</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
@@ -542,7 +542,7 @@
         <v>4.6875</v>
       </c>
       <c r="F4" t="n">
-        <v>0.0131</v>
+        <v>0.0095</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
@@ -573,7 +573,7 @@
         <v>4.734375</v>
       </c>
       <c r="F5" t="n">
-        <v>0.0065</v>
+        <v>0.0031</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
@@ -604,7 +604,7 @@
         <v>0.469727</v>
       </c>
       <c r="F6" t="n">
-        <v>0.7027</v>
+        <v>0.4156</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
@@ -635,7 +635,7 @@
         <v>0.472656</v>
       </c>
       <c r="F7" t="n">
-        <v>0.2817</v>
+        <v>0.1505</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
@@ -666,7 +666,7 @@
         <v>0.469727</v>
       </c>
       <c r="F8" t="n">
-        <v>0.7256</v>
+        <v>0.4288</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
@@ -697,7 +697,7 @@
         <v>0.942383</v>
       </c>
       <c r="F9" t="n">
-        <v>0.0327</v>
+        <v>0.019</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
@@ -729,7 +729,7 @@
         <v>0.942383</v>
       </c>
       <c r="F10" t="n">
-        <v>0.1283</v>
+        <v>0.07489999999999999</v>
       </c>
       <c r="G10" t="inlineStr">
         <is>
@@ -761,7 +761,7 @@
         <v>4.871094</v>
       </c>
       <c r="F11" t="n">
-        <v>0.0052</v>
+        <v>0.0027</v>
       </c>
       <c r="G11" t="inlineStr">
         <is>
@@ -793,7 +793,7 @@
         <v>4.863281</v>
       </c>
       <c r="F12" t="n">
-        <v>0.0047</v>
+        <v>0.0024</v>
       </c>
       <c r="G12" t="inlineStr">
         <is>
@@ -825,7 +825,7 @@
         <v>0.958008</v>
       </c>
       <c r="F13" t="n">
-        <v>1.3413</v>
+        <v>0.768</v>
       </c>
       <c r="G13" t="inlineStr">
         <is>
@@ -857,7 +857,7 @@
         <v>0.963867</v>
       </c>
       <c r="F14" t="n">
-        <v>0.6691</v>
+        <v>0.3857</v>
       </c>
       <c r="G14" t="inlineStr">
         <is>
@@ -889,7 +889,7 @@
         <v>0.942383</v>
       </c>
       <c r="F15" t="n">
-        <v>1.5857</v>
+        <v>0.8761</v>
       </c>
       <c r="G15" t="inlineStr">
         <is>
@@ -921,7 +921,7 @@
         <v>1.422852</v>
       </c>
       <c r="F16" t="n">
-        <v>0.0395</v>
+        <v>0.0232</v>
       </c>
       <c r="G16" t="inlineStr">
         <is>
@@ -954,7 +954,7 @@
         <v>1.422852</v>
       </c>
       <c r="F17" t="n">
-        <v>0.1388</v>
+        <v>0.0857</v>
       </c>
       <c r="G17" t="inlineStr">
         <is>
@@ -987,7 +987,7 @@
         <v>5.007812</v>
       </c>
       <c r="F18" t="n">
-        <v>0.0049</v>
+        <v>0.0027</v>
       </c>
       <c r="G18" t="inlineStr">
         <is>
@@ -1020,7 +1020,7 @@
         <v>5.011719</v>
       </c>
       <c r="F19" t="n">
-        <v>0.0049</v>
+        <v>0.0025</v>
       </c>
       <c r="G19" t="inlineStr">
         <is>
@@ -1053,7 +1053,7 @@
         <v>2.391602</v>
       </c>
       <c r="F20" t="n">
-        <v>1.0782</v>
+        <v>0.6324</v>
       </c>
       <c r="G20" t="inlineStr">
         <is>
@@ -1086,7 +1086,7 @@
         <v>1.436523</v>
       </c>
       <c r="F21" t="n">
-        <v>0.7713</v>
+        <v>0.429</v>
       </c>
       <c r="G21" t="inlineStr">
         <is>
@@ -1119,7 +1119,7 @@
         <v>1.422852</v>
       </c>
       <c r="F22" t="n">
-        <v>2.3047</v>
+        <v>1.0737</v>
       </c>
       <c r="G22" t="inlineStr">
         <is>
@@ -1152,7 +1152,7 @@
         <v>1.911133</v>
       </c>
       <c r="F23" t="n">
-        <v>0.0536</v>
+        <v>0.0283</v>
       </c>
       <c r="G23" t="inlineStr">
         <is>
@@ -1186,7 +1186,7 @@
         <v>1.911133</v>
       </c>
       <c r="F24" t="n">
-        <v>0.1633</v>
+        <v>0.08749999999999999</v>
       </c>
       <c r="G24" t="inlineStr">
         <is>
@@ -1220,7 +1220,7 @@
         <v>4.851562</v>
       </c>
       <c r="F25" t="n">
-        <v>0.0048</v>
+        <v>0.003</v>
       </c>
       <c r="G25" t="inlineStr">
         <is>
@@ -1254,7 +1254,7 @@
         <v>4.992188</v>
       </c>
       <c r="F26" t="n">
-        <v>0.008200000000000001</v>
+        <v>0.0034</v>
       </c>
       <c r="G26" t="inlineStr">
         <is>
@@ -1288,7 +1288,7 @@
         <v>1.938477</v>
       </c>
       <c r="F27" t="n">
-        <v>1.7161</v>
+        <v>0.8928</v>
       </c>
       <c r="G27" t="inlineStr">
         <is>
@@ -1322,7 +1322,7 @@
         <v>1.975586</v>
       </c>
       <c r="F28" t="n">
-        <v>1.0419</v>
+        <v>0.5343</v>
       </c>
       <c r="G28" t="inlineStr">
         <is>
@@ -1356,7 +1356,7 @@
         <v>1.911133</v>
       </c>
       <c r="F29" t="n">
-        <v>5.1986</v>
+        <v>1.2049</v>
       </c>
       <c r="G29" t="inlineStr">
         <is>
@@ -1390,7 +1390,7 @@
         <v>0.02679</v>
       </c>
       <c r="F30" t="n">
-        <v>0.2921</v>
+        <v>0.0467</v>
       </c>
       <c r="G30" t="inlineStr">
         <is>
@@ -1421,7 +1421,7 @@
         <v>0.02679</v>
       </c>
       <c r="F31" t="n">
-        <v>1.4848</v>
+        <v>0.3162</v>
       </c>
       <c r="G31" t="inlineStr">
         <is>
@@ -1452,7 +1452,7 @@
         <v>0.527377</v>
       </c>
       <c r="F32" t="n">
-        <v>0.022</v>
+        <v>0.0064</v>
       </c>
       <c r="G32" t="inlineStr">
         <is>
@@ -1483,7 +1483,7 @@
         <v>0.527377</v>
       </c>
       <c r="F33" t="n">
-        <v>0.0344</v>
+        <v>0.007</v>
       </c>
       <c r="G33" t="inlineStr">
         <is>
@@ -1514,7 +1514,7 @@
         <v>0.027029</v>
       </c>
       <c r="F34" t="n">
-        <v>3.1821</v>
+        <v>0.7665</v>
       </c>
       <c r="G34" t="inlineStr">
         <is>
@@ -1545,7 +1545,7 @@
         <v>0.027127</v>
       </c>
       <c r="F35" t="n">
-        <v>2.0781</v>
+        <v>0.485</v>
       </c>
       <c r="G35" t="inlineStr">
         <is>
@@ -1576,7 +1576,7 @@
         <v>0.02679</v>
       </c>
       <c r="F36" t="n">
-        <v>2.5708</v>
+        <v>0.9560999999999999</v>
       </c>
       <c r="G36" t="inlineStr">
         <is>
@@ -1607,7 +1607,7 @@
         <v>0.053819</v>
       </c>
       <c r="F37" t="n">
-        <v>0.2502</v>
+        <v>0.0564</v>
       </c>
       <c r="G37" t="inlineStr">
         <is>
@@ -1639,7 +1639,7 @@
         <v>0.053899</v>
       </c>
       <c r="F38" t="n">
-        <v>1.0513</v>
+        <v>0.3378</v>
       </c>
       <c r="G38" t="inlineStr">
         <is>
@@ -1671,7 +1671,7 @@
         <v>0.875242</v>
       </c>
       <c r="F39" t="n">
-        <v>0.0162</v>
+        <v>0.0057</v>
       </c>
       <c r="G39" t="inlineStr">
         <is>
@@ -1703,7 +1703,7 @@
         <v>1.07105</v>
       </c>
       <c r="F40" t="n">
-        <v>0.0182</v>
+        <v>0.0055</v>
       </c>
       <c r="G40" t="inlineStr">
         <is>
@@ -1735,7 +1735,7 @@
         <v>0.053899</v>
       </c>
       <c r="F41" t="n">
-        <v>2.7499</v>
+        <v>1.0628</v>
       </c>
       <c r="G41" t="inlineStr">
         <is>
@@ -1767,7 +1767,7 @@
         <v>0.054019</v>
       </c>
       <c r="F42" t="n">
-        <v>1.9823</v>
+        <v>0.794</v>
       </c>
       <c r="G42" t="inlineStr">
         <is>
@@ -1799,7 +1799,7 @@
         <v>0.053819</v>
       </c>
       <c r="F43" t="n">
-        <v>4.4157</v>
+        <v>1.5114</v>
       </c>
       <c r="G43" t="inlineStr">
         <is>
@@ -1831,7 +1831,7 @@
         <v>0.080928</v>
       </c>
       <c r="F44" t="n">
-        <v>0.2358</v>
+        <v>0.06950000000000001</v>
       </c>
       <c r="G44" t="inlineStr">
         <is>
@@ -1864,7 +1864,7 @@
         <v>0.081027</v>
       </c>
       <c r="F45" t="n">
-        <v>0.7759</v>
+        <v>0.3585</v>
       </c>
       <c r="G45" t="inlineStr">
         <is>
@@ -1897,7 +1897,7 @@
         <v>1.055199</v>
       </c>
       <c r="F46" t="n">
-        <v>0.0108</v>
+        <v>0.0062</v>
       </c>
       <c r="G46" t="inlineStr">
         <is>
@@ -1930,7 +1930,7 @@
         <v>1.076201</v>
       </c>
       <c r="F47" t="n">
-        <v>0.0094</v>
+        <v>0.0043</v>
       </c>
       <c r="G47" t="inlineStr">
         <is>
@@ -1963,7 +1963,7 @@
         <v>0.833143</v>
       </c>
       <c r="F48" t="n">
-        <v>3.7845</v>
+        <v>1.5238</v>
       </c>
       <c r="G48" t="inlineStr">
         <is>
@@ -1996,7 +1996,7 @@
         <v>0.834553</v>
       </c>
       <c r="F49" t="n">
-        <v>1.4305</v>
+        <v>1.0182</v>
       </c>
       <c r="G49" t="inlineStr">
         <is>
@@ -2029,7 +2029,7 @@
         <v>0.08094700000000001</v>
       </c>
       <c r="F50" t="n">
-        <v>3.0532</v>
+        <v>2.0047</v>
       </c>
       <c r="G50" t="inlineStr">
         <is>
@@ -2062,7 +2062,7 @@
         <v>0.108056</v>
       </c>
       <c r="F51" t="n">
-        <v>0.1221</v>
+        <v>0.0866</v>
       </c>
       <c r="G51" t="inlineStr">
         <is>
@@ -2096,7 +2096,7 @@
         <v>0.10818</v>
       </c>
       <c r="F52" t="n">
-        <v>0.6183999999999999</v>
+        <v>0.3882</v>
       </c>
       <c r="G52" t="inlineStr">
         <is>
@@ -2130,7 +2130,7 @@
         <v>1.089651</v>
       </c>
       <c r="F53" t="n">
-        <v>0.0091</v>
+        <v>0.007900000000000001</v>
       </c>
       <c r="G53" t="inlineStr">
         <is>
@@ -2164,7 +2164,7 @@
         <v>1.082651</v>
       </c>
       <c r="F54" t="n">
-        <v>0.0089</v>
+        <v>0.0077</v>
       </c>
       <c r="G54" t="inlineStr">
         <is>
@@ -2198,7 +2198,7 @@
         <v>0.108056</v>
       </c>
       <c r="F55" t="n">
-        <v>3.2998</v>
+        <v>1.9533</v>
       </c>
       <c r="G55" t="inlineStr">
         <is>
@@ -2232,7 +2232,7 @@
         <v>0.88572</v>
       </c>
       <c r="F56" t="n">
-        <v>1.5497</v>
+        <v>1.0479</v>
       </c>
       <c r="G56" t="inlineStr">
         <is>
@@ -2266,7 +2266,7 @@
         <v>0.108056</v>
       </c>
       <c r="F57" t="n">
-        <v>3.0202</v>
+        <v>1.9848</v>
       </c>
       <c r="G57" t="inlineStr">
         <is>
@@ -2300,7 +2300,7 @@
         <v>0.499296</v>
       </c>
       <c r="F58" t="n">
-        <v>2.3524</v>
+        <v>1.6351</v>
       </c>
       <c r="G58" t="inlineStr">
         <is>
@@ -2331,7 +2331,7 @@
         <v>0.499296</v>
       </c>
       <c r="F59" t="n">
-        <v>2.4145</v>
+        <v>1.6205</v>
       </c>
       <c r="G59" t="inlineStr">
         <is>
@@ -2362,7 +2362,7 @@
         <v>9.988281000000001</v>
       </c>
       <c r="F60" t="n">
-        <v>0.0746</v>
+        <v>0.0569</v>
       </c>
       <c r="G60" t="inlineStr">
         <is>
@@ -2393,7 +2393,7 @@
         <v>10.064453</v>
       </c>
       <c r="F61" t="n">
-        <v>0.0868</v>
+        <v>0.0635</v>
       </c>
       <c r="G61" t="inlineStr">
         <is>
@@ -2424,7 +2424,7 @@
         <v>0.499296</v>
       </c>
       <c r="F62" t="n">
-        <v>3.6729</v>
+        <v>1.7501</v>
       </c>
       <c r="G62" t="inlineStr">
         <is>
@@ -2455,7 +2455,7 @@
         <v>0.499616</v>
       </c>
       <c r="F63" t="n">
-        <v>2.5356</v>
+        <v>0.96</v>
       </c>
       <c r="G63" t="inlineStr">
         <is>
@@ -2486,7 +2486,7 @@
         <v>0.499296</v>
       </c>
       <c r="F64" t="n">
-        <v>3.8633</v>
+        <v>1.8661</v>
       </c>
       <c r="G64" t="inlineStr">
         <is>
@@ -2517,7 +2517,7 @@
         <v>0.998684</v>
       </c>
       <c r="F65" t="n">
-        <v>3.7949</v>
+        <v>1.7189</v>
       </c>
       <c r="G65" t="inlineStr">
         <is>
@@ -2549,7 +2549,7 @@
         <v>0.998684</v>
       </c>
       <c r="F66" t="n">
-        <v>2.9021</v>
+        <v>1.665</v>
       </c>
       <c r="G66" t="inlineStr">
         <is>
@@ -2581,7 +2581,7 @@
         <v>10.019196</v>
       </c>
       <c r="F67" t="n">
-        <v>0.1231</v>
+        <v>0.0641</v>
       </c>
       <c r="G67" t="inlineStr">
         <is>
@@ -2613,7 +2613,7 @@
         <v>10.059732</v>
       </c>
       <c r="F68" t="n">
-        <v>0.107</v>
+        <v>0.0593</v>
       </c>
       <c r="G68" t="inlineStr">
         <is>
@@ -2645,7 +2645,7 @@
         <v>1.499331</v>
       </c>
       <c r="F69" t="n">
-        <v>6.036</v>
+        <v>3.3113</v>
       </c>
       <c r="G69" t="inlineStr">
         <is>
@@ -2677,7 +2677,7 @@
         <v>1.00018</v>
       </c>
       <c r="F70" t="n">
-        <v>2.5336</v>
+        <v>1.4597</v>
       </c>
       <c r="G70" t="inlineStr">
         <is>
@@ -2709,7 +2709,7 @@
         <v>0.998684</v>
       </c>
       <c r="F71" t="n">
-        <v>4.5767</v>
+        <v>2.5192</v>
       </c>
       <c r="G71" t="inlineStr">
         <is>
@@ -2741,7 +2741,7 @@
         <v>1.498185</v>
       </c>
       <c r="F72" t="n">
-        <v>4.0675</v>
+        <v>1.8345</v>
       </c>
       <c r="G72" t="inlineStr">
         <is>
@@ -2774,7 +2774,7 @@
         <v>1.498185</v>
       </c>
       <c r="F73" t="n">
-        <v>3.0636</v>
+        <v>1.7919</v>
       </c>
       <c r="G73" t="inlineStr">
         <is>
@@ -2807,7 +2807,7 @@
         <v>10.022339</v>
       </c>
       <c r="F74" t="n">
-        <v>0.08160000000000001</v>
+        <v>0.0554</v>
       </c>
       <c r="G74" t="inlineStr">
         <is>
@@ -2840,7 +2840,7 @@
         <v>10.055605</v>
       </c>
       <c r="F75" t="n">
-        <v>0.1081</v>
+        <v>0.0594</v>
       </c>
       <c r="G75" t="inlineStr">
         <is>
@@ -2873,7 +2873,7 @@
         <v>3.998016</v>
       </c>
       <c r="F76" t="n">
-        <v>8.188499999999999</v>
+        <v>4.3469</v>
       </c>
       <c r="G76" t="inlineStr">
         <is>
@@ -2906,7 +2906,7 @@
         <v>6.999811</v>
       </c>
       <c r="F77" t="n">
-        <v>3.5016</v>
+        <v>1.7743</v>
       </c>
       <c r="G77" t="inlineStr">
         <is>
@@ -2939,7 +2939,7 @@
         <v>1.498507</v>
       </c>
       <c r="F78" t="n">
-        <v>4.907</v>
+        <v>3.2596</v>
       </c>
       <c r="G78" t="inlineStr">
         <is>
@@ -2972,7 +2972,7 @@
         <v>1.997801</v>
       </c>
       <c r="F79" t="n">
-        <v>4.607</v>
+        <v>2.0182</v>
       </c>
       <c r="G79" t="inlineStr">
         <is>
@@ -3006,7 +3006,7 @@
         <v>1.997801</v>
       </c>
       <c r="F80" t="n">
-        <v>6.8455</v>
+        <v>1.7452</v>
       </c>
       <c r="G80" t="inlineStr">
         <is>
@@ -3040,7 +3040,7 @@
         <v>10.009598</v>
       </c>
       <c r="F81" t="n">
-        <v>0.2411</v>
+        <v>0.0585</v>
       </c>
       <c r="G81" t="inlineStr">
         <is>
@@ -3074,7 +3074,7 @@
         <v>10.011873</v>
       </c>
       <c r="F82" t="n">
-        <v>0.2509</v>
+        <v>0.0611</v>
       </c>
       <c r="G82" t="inlineStr">
         <is>
@@ -3108,7 +3108,7 @@
         <v>4.997678</v>
       </c>
       <c r="F83" t="n">
-        <v>12.3664</v>
+        <v>4.3094</v>
       </c>
       <c r="G83" t="inlineStr">
         <is>
@@ -3142,7 +3142,7 @@
         <v>5.497547</v>
       </c>
       <c r="F84" t="n">
-        <v>6.1723</v>
+        <v>1.9097</v>
       </c>
       <c r="G84" t="inlineStr">
         <is>
@@ -3176,7 +3176,7 @@
         <v>1.997874</v>
       </c>
       <c r="F85" t="n">
-        <v>5.681</v>
+        <v>3.0629</v>
       </c>
       <c r="G85" t="inlineStr">
         <is>

</xml_diff>